<commit_message>
2026 03 20 001
1. 셋팅값 수정안 추가 - 주석처리함. 아직 테스트 못함.
2. 검사 before 40 -> 20초 수정
</commit_message>
<xml_diff>
--- a/마련 셋업.xlsx
+++ b/마련 셋업.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="20417"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{989668E9-9272-422C-AFED-B324C8CCCA5D}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0A673ECE-C574-4C4E-A502-737AE5430A41}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="8910" windowHeight="10845" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="502" uniqueCount="315">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="505" uniqueCount="317">
   <si>
     <t>순번</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -1317,6 +1317,20 @@
   </si>
   <si>
     <t>충전이 precharge1만 되고 멈춰서 마지막 전압값이 900mV 인경우가 있음. -&gt; 불량처리</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve">    CMD = "SEQ:STEP:DEF 1,1,PRECHARGE," + cPrechargeTime + ",1.0,2.0\n";
+    CMD += "SEQ:TEST:DEF 1,1,1,VOLT_GE,1.2,BEFORE,20,NEXT\n";
+    CMD += "SEQ:STEP:DEF 1,2,PRECHARGE2," + cTime + "," + cCurr + "," + cVolt + "\n";
+    CMD += "SEQ:TEST:DEF 1,2,1,CURR_LE,0.01,BEFORE,20,FAIL\n";
+    CMD += "SEQ:TEST:DEF 1,2,2,VOLT_LE,0.1,BEFORE,20,FAIL\n";
+    //* 2026 03 20 후에 테스트 필요
+    //CMD += "SEQ:TEST:DEF 1,2,3,CURR_LE,0.2,AFTER,20,NEXT \n";</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>셋팅 변경 후 테스트 필요</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -1731,7 +1745,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="130">
+  <cellXfs count="135">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" indent="1"/>
@@ -2040,6 +2054,12 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="176" fontId="0" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -2075,6 +2095,15 @@
     </xf>
     <xf numFmtId="176" fontId="3" fillId="4" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="6" fillId="2" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="6" fillId="2" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2366,12 +2395,12 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B2" s="118" t="s">
+      <c r="B2" s="120" t="s">
         <v>14</v>
       </c>
-      <c r="C2" s="118"/>
-      <c r="D2" s="118"/>
-      <c r="E2" s="118"/>
+      <c r="C2" s="120"/>
+      <c r="D2" s="120"/>
+      <c r="E2" s="120"/>
     </row>
     <row r="3" spans="2:5" ht="17.25" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="4" spans="2:5" s="3" customFormat="1" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
@@ -2389,12 +2418,12 @@
       </c>
     </row>
     <row r="5" spans="2:5" s="3" customFormat="1" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B5" s="119" t="s">
+      <c r="B5" s="121" t="s">
         <v>95</v>
       </c>
-      <c r="C5" s="120"/>
-      <c r="D5" s="120"/>
-      <c r="E5" s="121"/>
+      <c r="C5" s="122"/>
+      <c r="D5" s="122"/>
+      <c r="E5" s="123"/>
     </row>
     <row r="6" spans="2:5" s="3" customFormat="1" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B6" s="50" t="s">
@@ -2465,12 +2494,12 @@
       <c r="E11" s="7"/>
     </row>
     <row r="12" spans="2:5" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B12" s="119" t="s">
+      <c r="B12" s="121" t="s">
         <v>96</v>
       </c>
-      <c r="C12" s="120"/>
-      <c r="D12" s="120"/>
-      <c r="E12" s="121"/>
+      <c r="C12" s="122"/>
+      <c r="D12" s="122"/>
+      <c r="E12" s="123"/>
     </row>
     <row r="13" spans="2:5" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B13" s="50" t="s">
@@ -2544,12 +2573,12 @@
       <c r="H20" s="49"/>
     </row>
     <row r="23" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B23" s="118" t="s">
+      <c r="B23" s="120" t="s">
         <v>20</v>
       </c>
-      <c r="C23" s="118"/>
-      <c r="D23" s="118"/>
-      <c r="E23" s="118"/>
+      <c r="C23" s="120"/>
+      <c r="D23" s="120"/>
+      <c r="E23" s="120"/>
     </row>
     <row r="24" spans="2:8" ht="17.25" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="25" spans="2:8" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
@@ -2605,7 +2634,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B66418C2-2F25-4DF5-AD93-3985FBAF3208}">
-  <dimension ref="B1:F189"/>
+  <dimension ref="B1:F198"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="3" customWidth="1"/>
@@ -2635,11 +2664,11 @@
     <row r="3" spans="2:6" ht="24" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B3" s="55"/>
       <c r="C3" s="60"/>
-      <c r="D3" s="126" t="s">
+      <c r="D3" s="128" t="s">
         <v>66</v>
       </c>
-      <c r="E3" s="126"/>
-      <c r="F3" s="127"/>
+      <c r="E3" s="128"/>
+      <c r="F3" s="129"/>
     </row>
     <row r="4" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="B4" s="33">
@@ -2672,13 +2701,13 @@
       <c r="F5" s="9"/>
     </row>
     <row r="6" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
-      <c r="B6" s="124">
+      <c r="B6" s="126">
         <v>3</v>
       </c>
       <c r="C6" s="61" t="s">
         <v>130</v>
       </c>
-      <c r="D6" s="122">
+      <c r="D6" s="124">
         <v>45604</v>
       </c>
       <c r="E6" s="24" t="s">
@@ -2687,11 +2716,11 @@
       <c r="F6" s="16"/>
     </row>
     <row r="7" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
-      <c r="B7" s="125"/>
+      <c r="B7" s="127"/>
       <c r="C7" s="61" t="s">
         <v>130</v>
       </c>
-      <c r="D7" s="123"/>
+      <c r="D7" s="125"/>
       <c r="E7" s="24" t="s">
         <v>24</v>
       </c>
@@ -3178,11 +3207,11 @@
     <row r="38" spans="2:6" ht="25.5" hidden="1" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B38" s="56"/>
       <c r="C38" s="63"/>
-      <c r="D38" s="128" t="s">
+      <c r="D38" s="130" t="s">
         <v>67</v>
       </c>
-      <c r="E38" s="128"/>
-      <c r="F38" s="129"/>
+      <c r="E38" s="130"/>
+      <c r="F38" s="131"/>
     </row>
     <row r="39" spans="2:6" ht="17.25" hidden="1" thickTop="1" x14ac:dyDescent="0.3">
       <c r="B39" s="40">
@@ -4343,11 +4372,11 @@
     <row r="113" spans="2:6" ht="18" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B113" s="56"/>
       <c r="C113" s="63"/>
-      <c r="D113" s="128" t="s">
+      <c r="D113" s="130" t="s">
         <v>180</v>
       </c>
-      <c r="E113" s="128"/>
-      <c r="F113" s="129"/>
+      <c r="E113" s="130"/>
+      <c r="F113" s="131"/>
     </row>
     <row r="114" spans="2:6" ht="17.25" thickTop="1" x14ac:dyDescent="0.3">
       <c r="B114" s="67">
@@ -5516,26 +5545,99 @@
       </c>
       <c r="F186" s="16"/>
     </row>
-    <row r="187" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B187" s="32"/>
-      <c r="C187" s="62"/>
-      <c r="D187" s="31"/>
-      <c r="E187" s="22"/>
-      <c r="F187" s="16"/>
+    <row r="187" spans="2:6" ht="132" x14ac:dyDescent="0.3">
+      <c r="B187" s="132">
+        <v>147</v>
+      </c>
+      <c r="C187" s="84" t="s">
+        <v>131</v>
+      </c>
+      <c r="D187" s="85">
+        <v>46101</v>
+      </c>
+      <c r="E187" s="133" t="s">
+        <v>315</v>
+      </c>
+      <c r="F187" s="134" t="s">
+        <v>316</v>
+      </c>
     </row>
     <row r="188" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B188" s="32"/>
+      <c r="B188" s="119"/>
       <c r="C188" s="62"/>
-      <c r="D188" s="31"/>
-      <c r="E188" s="22"/>
+      <c r="D188" s="118"/>
+      <c r="E188" s="26"/>
       <c r="F188" s="16"/>
     </row>
-    <row r="189" spans="2:6" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B189" s="41"/>
-      <c r="C189" s="64"/>
-      <c r="D189" s="11"/>
-      <c r="E189" s="23"/>
-      <c r="F189" s="17"/>
+    <row r="189" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B189" s="119"/>
+      <c r="C189" s="62"/>
+      <c r="D189" s="118"/>
+      <c r="E189" s="26"/>
+      <c r="F189" s="16"/>
+    </row>
+    <row r="190" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B190" s="119"/>
+      <c r="C190" s="62"/>
+      <c r="D190" s="118"/>
+      <c r="E190" s="26"/>
+      <c r="F190" s="16"/>
+    </row>
+    <row r="191" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B191" s="119"/>
+      <c r="C191" s="62"/>
+      <c r="D191" s="118"/>
+      <c r="E191" s="26"/>
+      <c r="F191" s="16"/>
+    </row>
+    <row r="192" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B192" s="119"/>
+      <c r="C192" s="62"/>
+      <c r="D192" s="118"/>
+      <c r="E192" s="26"/>
+      <c r="F192" s="16"/>
+    </row>
+    <row r="193" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B193" s="119"/>
+      <c r="C193" s="62"/>
+      <c r="D193" s="118"/>
+      <c r="E193" s="26"/>
+      <c r="F193" s="16"/>
+    </row>
+    <row r="194" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B194" s="119"/>
+      <c r="C194" s="62"/>
+      <c r="D194" s="118"/>
+      <c r="E194" s="26"/>
+      <c r="F194" s="16"/>
+    </row>
+    <row r="195" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B195" s="119"/>
+      <c r="C195" s="62"/>
+      <c r="D195" s="118"/>
+      <c r="E195" s="26"/>
+      <c r="F195" s="16"/>
+    </row>
+    <row r="196" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B196" s="32"/>
+      <c r="C196" s="62"/>
+      <c r="D196" s="31"/>
+      <c r="E196" s="22"/>
+      <c r="F196" s="16"/>
+    </row>
+    <row r="197" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B197" s="32"/>
+      <c r="C197" s="62"/>
+      <c r="D197" s="31"/>
+      <c r="E197" s="22"/>
+      <c r="F197" s="16"/>
+    </row>
+    <row r="198" spans="2:6" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B198" s="41"/>
+      <c r="C198" s="64"/>
+      <c r="D198" s="11"/>
+      <c r="E198" s="23"/>
+      <c r="F198" s="17"/>
     </row>
   </sheetData>
   <mergeCells count="5">

</xml_diff>